<commit_message>
Excel File Update (wrong short_answer query is WIP)
</commit_message>
<xml_diff>
--- a/rag/evaluation/Annotations-flan-t5-large.xlsx
+++ b/rag/evaluation/Annotations-flan-t5-large.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macos/Desktop/nlp-hw1/rag/evaluation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A739418-3C34-BC49-A881-4A031DDF8A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A863584E-8D08-3949-968A-B48C6F7B9903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1759" uniqueCount="1390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1760" uniqueCount="1391">
   <si>
     <t>query_id</t>
   </si>
@@ -4190,13 +4190,23 @@
   </si>
   <si>
     <t>Curtis Emerson LeMay</t>
+  </si>
+  <si>
+    <t>?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4205,12 +4215,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -4225,9 +4247,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4535,6 +4564,7 @@
   <dimension ref="A1:I251"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="53.5" style="1" customWidth="1"/>
     <col min="3" max="3" width="16.1640625" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" customWidth="1"/>
@@ -4595,6 +4625,9 @@
       <c r="H2">
         <v>1</v>
       </c>
+      <c r="I2" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -4621,6 +4654,9 @@
       <c r="H3">
         <v>1</v>
       </c>
+      <c r="I3" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -4647,6 +4683,9 @@
       <c r="H4">
         <v>1</v>
       </c>
+      <c r="I4" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -4673,6 +4712,9 @@
       <c r="H5">
         <v>0</v>
       </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -4699,6 +4741,9 @@
       <c r="H6">
         <v>1</v>
       </c>
+      <c r="I6" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -4725,6 +4770,9 @@
       <c r="H7">
         <v>1</v>
       </c>
+      <c r="I7" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -4751,6 +4799,9 @@
       <c r="H8">
         <v>1</v>
       </c>
+      <c r="I8" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -4777,6 +4828,9 @@
       <c r="H9">
         <v>1</v>
       </c>
+      <c r="I9" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -4803,6 +4857,9 @@
       <c r="H10">
         <v>1</v>
       </c>
+      <c r="I10" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -4829,6 +4886,9 @@
       <c r="H11">
         <v>1</v>
       </c>
+      <c r="I11" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -4855,6 +4915,9 @@
       <c r="H12">
         <v>1</v>
       </c>
+      <c r="I12" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -4881,6 +4944,9 @@
       <c r="H13">
         <v>0</v>
       </c>
+      <c r="I13" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -4907,6 +4973,9 @@
       <c r="H14">
         <v>0</v>
       </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -4933,6 +5002,9 @@
       <c r="H15">
         <v>1</v>
       </c>
+      <c r="I15" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -4959,8 +5031,11 @@
       <c r="H16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I16" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -4985,8 +5060,11 @@
       <c r="H17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>100</v>
       </c>
@@ -5011,8 +5089,11 @@
       <c r="H18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I18" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>105</v>
       </c>
@@ -5037,8 +5118,11 @@
       <c r="H19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I19" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>110</v>
       </c>
@@ -5063,8 +5147,11 @@
       <c r="H20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I20" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>115</v>
       </c>
@@ -5089,8 +5176,11 @@
       <c r="H21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>120</v>
       </c>
@@ -5115,8 +5205,11 @@
       <c r="H22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I22" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>125</v>
       </c>
@@ -5141,8 +5234,11 @@
       <c r="H23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I23" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>130</v>
       </c>
@@ -5167,8 +5263,11 @@
       <c r="H24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I24" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>136</v>
       </c>
@@ -5193,8 +5292,11 @@
       <c r="H25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I25" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>141</v>
       </c>
@@ -5219,8 +5321,11 @@
       <c r="H26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I26" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>146</v>
       </c>
@@ -5245,8 +5350,11 @@
       <c r="H27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I27" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>152</v>
       </c>
@@ -5271,8 +5379,11 @@
       <c r="H28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I28" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>158</v>
       </c>
@@ -5297,8 +5408,11 @@
       <c r="H29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+      <c r="I29" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>163</v>
       </c>
@@ -5323,8 +5437,11 @@
       <c r="H30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I30" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>169</v>
       </c>
@@ -5349,8 +5466,11 @@
       <c r="H31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I31" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>174</v>
       </c>
@@ -5375,8 +5495,11 @@
       <c r="H32">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I32" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>179</v>
       </c>
@@ -5401,8 +5524,11 @@
       <c r="H33">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I33" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>185</v>
       </c>
@@ -5427,8 +5553,11 @@
       <c r="H34">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I34" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>191</v>
       </c>
@@ -5453,8 +5582,11 @@
       <c r="H35">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I35" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>197</v>
       </c>
@@ -5479,8 +5611,11 @@
       <c r="H36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I36" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>202</v>
       </c>
@@ -5505,8 +5640,11 @@
       <c r="H37">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>206</v>
       </c>
@@ -5531,8 +5669,11 @@
       <c r="H38">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+      <c r="I38" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>211</v>
       </c>
@@ -5557,8 +5698,11 @@
       <c r="H39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I39" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>217</v>
       </c>
@@ -5583,8 +5727,11 @@
       <c r="H40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I40" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>223</v>
       </c>
@@ -5609,8 +5756,11 @@
       <c r="H41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I41" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>229</v>
       </c>
@@ -5633,10 +5783,13 @@
         <v>14</v>
       </c>
       <c r="H42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="I42" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>234</v>
       </c>
@@ -5661,8 +5814,11 @@
       <c r="H43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I43" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>240</v>
       </c>
@@ -5687,8 +5843,11 @@
       <c r="H44">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I44" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>245</v>
       </c>
@@ -5713,8 +5872,11 @@
       <c r="H45">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I45" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>250</v>
       </c>
@@ -5739,8 +5901,11 @@
       <c r="H46">
         <v>1</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I46" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>256</v>
       </c>
@@ -5765,8 +5930,11 @@
       <c r="H47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I47" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>261</v>
       </c>
@@ -5791,8 +5959,11 @@
       <c r="H48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I48" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>267</v>
       </c>
@@ -5817,8 +5988,11 @@
       <c r="H49">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I49" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>273</v>
       </c>
@@ -5843,8 +6017,11 @@
       <c r="H50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I50" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>279</v>
       </c>
@@ -5869,8 +6046,11 @@
       <c r="H51">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I51" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>285</v>
       </c>
@@ -5895,8 +6075,11 @@
       <c r="H52">
         <v>1</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I52" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>291</v>
       </c>
@@ -5921,8 +6104,11 @@
       <c r="H53">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I53" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>297</v>
       </c>
@@ -5947,8 +6133,11 @@
       <c r="H54">
         <v>1</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I54" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>302</v>
       </c>
@@ -5973,8 +6162,11 @@
       <c r="H55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I55" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>308</v>
       </c>
@@ -5999,8 +6191,11 @@
       <c r="H56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I56" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>314</v>
       </c>
@@ -6025,8 +6220,11 @@
       <c r="H57">
         <v>1</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I57" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>320</v>
       </c>
@@ -6051,8 +6249,11 @@
       <c r="H58">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I58" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>325</v>
       </c>
@@ -6077,8 +6278,11 @@
       <c r="H59">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I59" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>330</v>
       </c>
@@ -6103,8 +6307,11 @@
       <c r="H60">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I60" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>335</v>
       </c>
@@ -6129,8 +6336,11 @@
       <c r="H61">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I61" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>341</v>
       </c>
@@ -6155,8 +6365,11 @@
       <c r="H62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I62" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>347</v>
       </c>
@@ -6181,8 +6394,11 @@
       <c r="H63">
         <v>1</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I63" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>352</v>
       </c>
@@ -6207,8 +6423,11 @@
       <c r="H64">
         <v>1</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" ht="96" x14ac:dyDescent="0.2">
+      <c r="I64" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>358</v>
       </c>
@@ -6233,8 +6452,11 @@
       <c r="H65">
         <v>1</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I65" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>363</v>
       </c>
@@ -6259,8 +6481,11 @@
       <c r="H66">
         <v>1</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I66" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>369</v>
       </c>
@@ -6285,8 +6510,11 @@
       <c r="H67">
         <v>1</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I67" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>374</v>
       </c>
@@ -6311,8 +6539,11 @@
       <c r="H68">
         <v>1</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I68" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>379</v>
       </c>
@@ -6337,8 +6568,11 @@
       <c r="H69">
         <v>1</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I69" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>385</v>
       </c>
@@ -6363,8 +6597,11 @@
       <c r="H70">
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+      <c r="I70" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>391</v>
       </c>
@@ -6389,8 +6626,11 @@
       <c r="H71">
         <v>1</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I71" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>397</v>
       </c>
@@ -6415,8 +6655,11 @@
       <c r="H72">
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I72" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>403</v>
       </c>
@@ -6441,8 +6684,11 @@
       <c r="H73">
         <v>1</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I73" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>409</v>
       </c>
@@ -6467,8 +6713,11 @@
       <c r="H74">
         <v>1</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I74" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>415</v>
       </c>
@@ -6493,8 +6742,11 @@
       <c r="H75">
         <v>1</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I75" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>421</v>
       </c>
@@ -6519,8 +6771,11 @@
       <c r="H76">
         <v>1</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I76" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>426</v>
       </c>
@@ -6545,8 +6800,11 @@
       <c r="H77">
         <v>1</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" ht="112" x14ac:dyDescent="0.2">
+      <c r="I77" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="112" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>431</v>
       </c>
@@ -6571,8 +6829,11 @@
       <c r="H78">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I78" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>437</v>
       </c>
@@ -6597,8 +6858,11 @@
       <c r="H79">
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I79" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>443</v>
       </c>
@@ -6623,8 +6887,11 @@
       <c r="H80">
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I80" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>449</v>
       </c>
@@ -6649,8 +6916,11 @@
       <c r="H81">
         <v>1</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I81" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>454</v>
       </c>
@@ -6675,8 +6945,11 @@
       <c r="H82">
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I82" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>460</v>
       </c>
@@ -6701,8 +6974,11 @@
       <c r="H83">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I83" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>466</v>
       </c>
@@ -6727,8 +7003,11 @@
       <c r="H84">
         <v>1</v>
       </c>
-    </row>
-    <row r="85" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I84" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>472</v>
       </c>
@@ -6753,8 +7032,11 @@
       <c r="H85">
         <v>1</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I85" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>477</v>
       </c>
@@ -6779,8 +7061,11 @@
       <c r="H86">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I86" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>483</v>
       </c>
@@ -6805,8 +7090,11 @@
       <c r="H87">
         <v>1</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I87" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>488</v>
       </c>
@@ -6831,8 +7119,11 @@
       <c r="H88">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I88" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>494</v>
       </c>
@@ -6857,8 +7148,11 @@
       <c r="H89">
         <v>1</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I89" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>499</v>
       </c>
@@ -6883,8 +7177,11 @@
       <c r="H90">
         <v>1</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I90" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>505</v>
       </c>
@@ -6909,8 +7206,11 @@
       <c r="H91">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+      <c r="I91" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>511</v>
       </c>
@@ -6933,10 +7233,13 @@
         <v>14</v>
       </c>
       <c r="H92">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="I92" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>517</v>
       </c>
@@ -6961,8 +7264,11 @@
       <c r="H93">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I93" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>523</v>
       </c>
@@ -6987,8 +7293,11 @@
       <c r="H94">
         <v>1</v>
       </c>
-    </row>
-    <row r="95" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I94" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>529</v>
       </c>
@@ -7013,8 +7322,11 @@
       <c r="H95">
         <v>1</v>
       </c>
-    </row>
-    <row r="96" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I95" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>535</v>
       </c>
@@ -7039,8 +7351,11 @@
       <c r="H96">
         <v>1</v>
       </c>
-    </row>
-    <row r="97" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I96" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>540</v>
       </c>
@@ -7065,8 +7380,11 @@
       <c r="H97">
         <v>1</v>
       </c>
-    </row>
-    <row r="98" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I97" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>546</v>
       </c>
@@ -7089,10 +7407,13 @@
         <v>14</v>
       </c>
       <c r="H98">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="I98" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>552</v>
       </c>
@@ -7117,8 +7438,11 @@
       <c r="H99">
         <v>1</v>
       </c>
-    </row>
-    <row r="100" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I99" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>558</v>
       </c>
@@ -7143,8 +7467,11 @@
       <c r="H100">
         <v>0</v>
       </c>
-    </row>
-    <row r="101" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I100" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>564</v>
       </c>
@@ -7169,8 +7496,11 @@
       <c r="H101">
         <v>1</v>
       </c>
-    </row>
-    <row r="102" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I101" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>569</v>
       </c>
@@ -7195,8 +7525,11 @@
       <c r="H102">
         <v>0</v>
       </c>
-    </row>
-    <row r="103" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I102" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>575</v>
       </c>
@@ -7221,8 +7554,11 @@
       <c r="H103">
         <v>1</v>
       </c>
-    </row>
-    <row r="104" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I103" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>581</v>
       </c>
@@ -7247,8 +7583,11 @@
       <c r="H104">
         <v>0</v>
       </c>
-    </row>
-    <row r="105" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I104" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>586</v>
       </c>
@@ -7273,8 +7612,11 @@
       <c r="H105">
         <v>1</v>
       </c>
-    </row>
-    <row r="106" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I105" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>590</v>
       </c>
@@ -7299,8 +7641,11 @@
       <c r="H106">
         <v>1</v>
       </c>
-    </row>
-    <row r="107" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I106" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>596</v>
       </c>
@@ -7325,8 +7670,11 @@
       <c r="H107">
         <v>0</v>
       </c>
-    </row>
-    <row r="108" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I107" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>602</v>
       </c>
@@ -7351,8 +7699,11 @@
       <c r="H108">
         <v>1</v>
       </c>
-    </row>
-    <row r="109" spans="1:8" ht="112" x14ac:dyDescent="0.2">
+      <c r="I108" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" ht="112" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>607</v>
       </c>
@@ -7377,8 +7728,11 @@
       <c r="H109">
         <v>0</v>
       </c>
-    </row>
-    <row r="110" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I109" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>613</v>
       </c>
@@ -7403,8 +7757,11 @@
       <c r="H110">
         <v>1</v>
       </c>
-    </row>
-    <row r="111" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I110" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>618</v>
       </c>
@@ -7429,8 +7786,11 @@
       <c r="H111">
         <v>1</v>
       </c>
-    </row>
-    <row r="112" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I111" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>623</v>
       </c>
@@ -7455,8 +7815,11 @@
       <c r="H112">
         <v>0</v>
       </c>
-    </row>
-    <row r="113" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I112" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>629</v>
       </c>
@@ -7481,8 +7844,11 @@
       <c r="H113">
         <v>1</v>
       </c>
-    </row>
-    <row r="114" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I113" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>633</v>
       </c>
@@ -7507,8 +7873,11 @@
       <c r="H114">
         <v>1</v>
       </c>
-    </row>
-    <row r="115" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I114" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>638</v>
       </c>
@@ -7533,8 +7902,11 @@
       <c r="H115">
         <v>0</v>
       </c>
-    </row>
-    <row r="116" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I115" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>644</v>
       </c>
@@ -7559,8 +7931,11 @@
       <c r="H116">
         <v>0</v>
       </c>
-    </row>
-    <row r="117" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I116" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>650</v>
       </c>
@@ -7585,8 +7960,11 @@
       <c r="H117">
         <v>1</v>
       </c>
-    </row>
-    <row r="118" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I117" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>656</v>
       </c>
@@ -7611,8 +7989,11 @@
       <c r="H118">
         <v>1</v>
       </c>
-    </row>
-    <row r="119" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I118" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>662</v>
       </c>
@@ -7637,8 +8018,11 @@
       <c r="H119">
         <v>0</v>
       </c>
-    </row>
-    <row r="120" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I119" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>668</v>
       </c>
@@ -7663,8 +8047,11 @@
       <c r="H120">
         <v>1</v>
       </c>
-    </row>
-    <row r="121" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I120" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>673</v>
       </c>
@@ -7689,8 +8076,11 @@
       <c r="H121">
         <v>1</v>
       </c>
-    </row>
-    <row r="122" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I121" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>679</v>
       </c>
@@ -7715,8 +8105,11 @@
       <c r="H122">
         <v>1</v>
       </c>
-    </row>
-    <row r="123" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I122" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>684</v>
       </c>
@@ -7741,8 +8134,11 @@
       <c r="H123">
         <v>0</v>
       </c>
-    </row>
-    <row r="124" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I123" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>690</v>
       </c>
@@ -7767,8 +8163,11 @@
       <c r="H124">
         <v>0</v>
       </c>
-    </row>
-    <row r="125" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I124" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>696</v>
       </c>
@@ -7793,8 +8192,11 @@
       <c r="H125">
         <v>0</v>
       </c>
-    </row>
-    <row r="126" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I125" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>702</v>
       </c>
@@ -7819,8 +8221,11 @@
       <c r="H126">
         <v>1</v>
       </c>
-    </row>
-    <row r="127" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I126" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>707</v>
       </c>
@@ -7845,8 +8250,11 @@
       <c r="H127">
         <v>0</v>
       </c>
-    </row>
-    <row r="128" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I127" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>713</v>
       </c>
@@ -7871,8 +8279,11 @@
       <c r="H128">
         <v>0</v>
       </c>
-    </row>
-    <row r="129" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I128" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>719</v>
       </c>
@@ -7897,8 +8308,11 @@
       <c r="H129">
         <v>1</v>
       </c>
-    </row>
-    <row r="130" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+      <c r="I129" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>723</v>
       </c>
@@ -7923,8 +8337,11 @@
       <c r="H130">
         <v>0</v>
       </c>
-    </row>
-    <row r="131" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I130" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>729</v>
       </c>
@@ -7949,8 +8366,11 @@
       <c r="H131">
         <v>1</v>
       </c>
-    </row>
-    <row r="132" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I131" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>735</v>
       </c>
@@ -7975,8 +8395,11 @@
       <c r="H132">
         <v>1</v>
       </c>
-    </row>
-    <row r="133" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I132" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>741</v>
       </c>
@@ -8001,8 +8424,11 @@
       <c r="H133">
         <v>1</v>
       </c>
-    </row>
-    <row r="134" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I133" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>747</v>
       </c>
@@ -8027,8 +8453,11 @@
       <c r="H134">
         <v>1</v>
       </c>
-    </row>
-    <row r="135" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I134" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>753</v>
       </c>
@@ -8053,8 +8482,11 @@
       <c r="H135">
         <v>1</v>
       </c>
-    </row>
-    <row r="136" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I135" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>758</v>
       </c>
@@ -8079,8 +8511,11 @@
       <c r="H136">
         <v>0</v>
       </c>
-    </row>
-    <row r="137" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I136" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>764</v>
       </c>
@@ -8105,8 +8540,11 @@
       <c r="H137">
         <v>1</v>
       </c>
-    </row>
-    <row r="138" spans="1:8" ht="96" x14ac:dyDescent="0.2">
+      <c r="I137" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>770</v>
       </c>
@@ -8131,8 +8569,11 @@
       <c r="H138">
         <v>1</v>
       </c>
-    </row>
-    <row r="139" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I138" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>776</v>
       </c>
@@ -8157,8 +8598,11 @@
       <c r="H139">
         <v>1</v>
       </c>
-    </row>
-    <row r="140" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I139" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>781</v>
       </c>
@@ -8183,8 +8627,11 @@
       <c r="H140">
         <v>0</v>
       </c>
-    </row>
-    <row r="141" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I140" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>787</v>
       </c>
@@ -8209,8 +8656,11 @@
       <c r="H141">
         <v>1</v>
       </c>
-    </row>
-    <row r="142" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I141" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>792</v>
       </c>
@@ -8235,8 +8685,11 @@
       <c r="H142">
         <v>1</v>
       </c>
-    </row>
-    <row r="143" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I142" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>796</v>
       </c>
@@ -8261,8 +8714,11 @@
       <c r="H143">
         <v>1</v>
       </c>
-    </row>
-    <row r="144" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I143" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>802</v>
       </c>
@@ -8287,8 +8743,11 @@
       <c r="H144">
         <v>1</v>
       </c>
-    </row>
-    <row r="145" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I144" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>808</v>
       </c>
@@ -8313,8 +8772,11 @@
       <c r="H145">
         <v>1</v>
       </c>
-    </row>
-    <row r="146" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I145" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>814</v>
       </c>
@@ -8339,8 +8801,11 @@
       <c r="H146">
         <v>1</v>
       </c>
-    </row>
-    <row r="147" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I146" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>820</v>
       </c>
@@ -8365,8 +8830,11 @@
       <c r="H147">
         <v>1</v>
       </c>
-    </row>
-    <row r="148" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I147" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>825</v>
       </c>
@@ -8391,8 +8859,11 @@
       <c r="H148">
         <v>0</v>
       </c>
-    </row>
-    <row r="149" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I148" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>831</v>
       </c>
@@ -8417,8 +8888,11 @@
       <c r="H149">
         <v>1</v>
       </c>
-    </row>
-    <row r="150" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I149" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>837</v>
       </c>
@@ -8443,8 +8917,11 @@
       <c r="H150">
         <v>1</v>
       </c>
-    </row>
-    <row r="151" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I150" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>843</v>
       </c>
@@ -8469,8 +8946,11 @@
       <c r="H151">
         <v>1</v>
       </c>
-    </row>
-    <row r="152" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I151" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>849</v>
       </c>
@@ -8495,8 +8975,11 @@
       <c r="H152">
         <v>0</v>
       </c>
-    </row>
-    <row r="153" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I152" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>855</v>
       </c>
@@ -8521,8 +9004,11 @@
       <c r="H153">
         <v>1</v>
       </c>
-    </row>
-    <row r="154" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I153" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>860</v>
       </c>
@@ -8547,8 +9033,11 @@
       <c r="H154">
         <v>0</v>
       </c>
-    </row>
-    <row r="155" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I154" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>866</v>
       </c>
@@ -8573,8 +9062,11 @@
       <c r="H155">
         <v>1</v>
       </c>
-    </row>
-    <row r="156" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I155" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>871</v>
       </c>
@@ -8599,8 +9091,11 @@
       <c r="H156">
         <v>0</v>
       </c>
-    </row>
-    <row r="157" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I156" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>877</v>
       </c>
@@ -8625,8 +9120,11 @@
       <c r="H157">
         <v>1</v>
       </c>
-    </row>
-    <row r="158" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I157" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>881</v>
       </c>
@@ -8651,8 +9149,11 @@
       <c r="H158">
         <v>0</v>
       </c>
-    </row>
-    <row r="159" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I158" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>886</v>
       </c>
@@ -8677,8 +9178,11 @@
       <c r="H159">
         <v>1</v>
       </c>
-    </row>
-    <row r="160" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I159" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>891</v>
       </c>
@@ -8703,8 +9207,11 @@
       <c r="H160">
         <v>1</v>
       </c>
-    </row>
-    <row r="161" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+      <c r="I160" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>896</v>
       </c>
@@ -8729,8 +9236,11 @@
       <c r="H161">
         <v>1</v>
       </c>
-    </row>
-    <row r="162" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I161" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>902</v>
       </c>
@@ -8755,8 +9265,11 @@
       <c r="H162">
         <v>1</v>
       </c>
-    </row>
-    <row r="163" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I162" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>907</v>
       </c>
@@ -8781,8 +9294,11 @@
       <c r="H163">
         <v>1</v>
       </c>
-    </row>
-    <row r="164" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I163" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>913</v>
       </c>
@@ -8807,8 +9323,11 @@
       <c r="H164">
         <v>1</v>
       </c>
-    </row>
-    <row r="165" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I164" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>919</v>
       </c>
@@ -8833,8 +9352,11 @@
       <c r="H165">
         <v>1</v>
       </c>
-    </row>
-    <row r="166" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I165" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>923</v>
       </c>
@@ -8859,8 +9381,11 @@
       <c r="H166">
         <v>1</v>
       </c>
-    </row>
-    <row r="167" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I166" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>929</v>
       </c>
@@ -8885,8 +9410,11 @@
       <c r="H167">
         <v>0</v>
       </c>
-    </row>
-    <row r="168" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I167" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>935</v>
       </c>
@@ -8911,8 +9439,11 @@
       <c r="H168">
         <v>0</v>
       </c>
-    </row>
-    <row r="169" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I168" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>941</v>
       </c>
@@ -8937,8 +9468,11 @@
       <c r="H169">
         <v>0</v>
       </c>
-    </row>
-    <row r="170" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I169" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>947</v>
       </c>
@@ -8963,8 +9497,11 @@
       <c r="H170">
         <v>1</v>
       </c>
-    </row>
-    <row r="171" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I170" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>952</v>
       </c>
@@ -8989,8 +9526,11 @@
       <c r="H171">
         <v>1</v>
       </c>
-    </row>
-    <row r="172" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I171" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>958</v>
       </c>
@@ -9015,8 +9555,11 @@
       <c r="H172">
         <v>1</v>
       </c>
-    </row>
-    <row r="173" spans="1:8" ht="96" x14ac:dyDescent="0.2">
+      <c r="I172" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>963</v>
       </c>
@@ -9041,8 +9584,11 @@
       <c r="H173">
         <v>1</v>
       </c>
-    </row>
-    <row r="174" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I173" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>969</v>
       </c>
@@ -9067,8 +9613,11 @@
       <c r="H174">
         <v>1</v>
       </c>
-    </row>
-    <row r="175" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I174" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>975</v>
       </c>
@@ -9093,8 +9642,11 @@
       <c r="H175">
         <v>1</v>
       </c>
-    </row>
-    <row r="176" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I175" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>980</v>
       </c>
@@ -9119,8 +9671,11 @@
       <c r="H176">
         <v>1</v>
       </c>
-    </row>
-    <row r="177" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+      <c r="I176" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>986</v>
       </c>
@@ -9145,8 +9700,11 @@
       <c r="H177">
         <v>1</v>
       </c>
-    </row>
-    <row r="178" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I177" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>992</v>
       </c>
@@ -9171,8 +9729,11 @@
       <c r="H178">
         <v>1</v>
       </c>
-    </row>
-    <row r="179" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I178" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>998</v>
       </c>
@@ -9197,8 +9758,11 @@
       <c r="H179">
         <v>1</v>
       </c>
-    </row>
-    <row r="180" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I179" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>1003</v>
       </c>
@@ -9223,8 +9787,11 @@
       <c r="H180">
         <v>1</v>
       </c>
-    </row>
-    <row r="181" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I180" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>1008</v>
       </c>
@@ -9249,8 +9816,11 @@
       <c r="H181">
         <v>1</v>
       </c>
-    </row>
-    <row r="182" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I181" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>1013</v>
       </c>
@@ -9275,8 +9845,11 @@
       <c r="H182">
         <v>0</v>
       </c>
-    </row>
-    <row r="183" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I182" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>1019</v>
       </c>
@@ -9301,8 +9874,11 @@
       <c r="H183">
         <v>0</v>
       </c>
-    </row>
-    <row r="184" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I183" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>1025</v>
       </c>
@@ -9327,8 +9903,11 @@
       <c r="H184">
         <v>1</v>
       </c>
-    </row>
-    <row r="185" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I184" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>1029</v>
       </c>
@@ -9351,10 +9930,13 @@
         <v>14</v>
       </c>
       <c r="H185">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="186" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="I185" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>1034</v>
       </c>
@@ -9379,8 +9961,11 @@
       <c r="H186">
         <v>1</v>
       </c>
-    </row>
-    <row r="187" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I186" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>1039</v>
       </c>
@@ -9405,8 +9990,11 @@
       <c r="H187">
         <v>1</v>
       </c>
-    </row>
-    <row r="188" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I187" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>1045</v>
       </c>
@@ -9431,8 +10019,11 @@
       <c r="H188">
         <v>1</v>
       </c>
-    </row>
-    <row r="189" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I188" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>1050</v>
       </c>
@@ -9457,8 +10048,11 @@
       <c r="H189">
         <v>1</v>
       </c>
-    </row>
-    <row r="190" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I189" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>1055</v>
       </c>
@@ -9483,8 +10077,11 @@
       <c r="H190">
         <v>0</v>
       </c>
-    </row>
-    <row r="191" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I190" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>1060</v>
       </c>
@@ -9509,8 +10106,11 @@
       <c r="H191">
         <v>1</v>
       </c>
-    </row>
-    <row r="192" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I191" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>1066</v>
       </c>
@@ -9535,8 +10135,11 @@
       <c r="H192">
         <v>1</v>
       </c>
-    </row>
-    <row r="193" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I192" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>1071</v>
       </c>
@@ -9561,8 +10164,11 @@
       <c r="H193">
         <v>1</v>
       </c>
-    </row>
-    <row r="194" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I193" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>1075</v>
       </c>
@@ -9587,8 +10193,11 @@
       <c r="H194">
         <v>1</v>
       </c>
-    </row>
-    <row r="195" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I194" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>1081</v>
       </c>
@@ -9613,8 +10222,11 @@
       <c r="H195">
         <v>1</v>
       </c>
-    </row>
-    <row r="196" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I195" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>1085</v>
       </c>
@@ -9639,8 +10251,11 @@
       <c r="H196">
         <v>1</v>
       </c>
-    </row>
-    <row r="197" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I196" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>1091</v>
       </c>
@@ -9665,8 +10280,11 @@
       <c r="H197">
         <v>0</v>
       </c>
-    </row>
-    <row r="198" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I197" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>1097</v>
       </c>
@@ -9691,8 +10309,11 @@
       <c r="H198">
         <v>1</v>
       </c>
-    </row>
-    <row r="199" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I198" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>1101</v>
       </c>
@@ -9717,8 +10338,11 @@
       <c r="H199">
         <v>1</v>
       </c>
-    </row>
-    <row r="200" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I199" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>1107</v>
       </c>
@@ -9743,8 +10367,11 @@
       <c r="H200">
         <v>0</v>
       </c>
-    </row>
-    <row r="201" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I200" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>1112</v>
       </c>
@@ -9769,8 +10396,11 @@
       <c r="H201">
         <v>1</v>
       </c>
-    </row>
-    <row r="202" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I201" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>1118</v>
       </c>
@@ -9795,8 +10425,11 @@
       <c r="H202">
         <v>0</v>
       </c>
-    </row>
-    <row r="203" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I202" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>1124</v>
       </c>
@@ -9821,8 +10454,11 @@
       <c r="H203">
         <v>1</v>
       </c>
-    </row>
-    <row r="204" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I203" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>1129</v>
       </c>
@@ -9847,8 +10483,11 @@
       <c r="H204">
         <v>1</v>
       </c>
-    </row>
-    <row r="205" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I204" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>1134</v>
       </c>
@@ -9873,8 +10512,11 @@
       <c r="H205">
         <v>1</v>
       </c>
-    </row>
-    <row r="206" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I205" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>1139</v>
       </c>
@@ -9899,8 +10541,11 @@
       <c r="H206">
         <v>1</v>
       </c>
-    </row>
-    <row r="207" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I206" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>1143</v>
       </c>
@@ -9925,8 +10570,11 @@
       <c r="H207">
         <v>1</v>
       </c>
-    </row>
-    <row r="208" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I207" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>1148</v>
       </c>
@@ -9951,8 +10599,11 @@
       <c r="H208">
         <v>1</v>
       </c>
-    </row>
-    <row r="209" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+      <c r="I208" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>1153</v>
       </c>
@@ -9977,8 +10628,11 @@
       <c r="H209">
         <v>1</v>
       </c>
-    </row>
-    <row r="210" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I209" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>1159</v>
       </c>
@@ -10003,8 +10657,11 @@
       <c r="H210">
         <v>1</v>
       </c>
-    </row>
-    <row r="211" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I210" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>1164</v>
       </c>
@@ -10029,8 +10686,11 @@
       <c r="H211">
         <v>1</v>
       </c>
-    </row>
-    <row r="212" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I211" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>1169</v>
       </c>
@@ -10055,8 +10715,11 @@
       <c r="H212">
         <v>1</v>
       </c>
-    </row>
-    <row r="213" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I212" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>1174</v>
       </c>
@@ -10081,8 +10744,11 @@
       <c r="H213">
         <v>1</v>
       </c>
-    </row>
-    <row r="214" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I213" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>1179</v>
       </c>
@@ -10107,8 +10773,11 @@
       <c r="H214">
         <v>1</v>
       </c>
-    </row>
-    <row r="215" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I214" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>1184</v>
       </c>
@@ -10133,8 +10802,11 @@
       <c r="H215">
         <v>1</v>
       </c>
-    </row>
-    <row r="216" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I215" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>1190</v>
       </c>
@@ -10159,8 +10831,11 @@
       <c r="H216">
         <v>1</v>
       </c>
-    </row>
-    <row r="217" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I216" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>1196</v>
       </c>
@@ -10185,8 +10860,11 @@
       <c r="H217">
         <v>0</v>
       </c>
-    </row>
-    <row r="218" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I217" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>1202</v>
       </c>
@@ -10211,8 +10889,11 @@
       <c r="H218">
         <v>1</v>
       </c>
-    </row>
-    <row r="219" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I218" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>1208</v>
       </c>
@@ -10237,8 +10918,11 @@
       <c r="H219">
         <v>1</v>
       </c>
-    </row>
-    <row r="220" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I219" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>1214</v>
       </c>
@@ -10263,8 +10947,11 @@
       <c r="H220">
         <v>1</v>
       </c>
-    </row>
-    <row r="221" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I220" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>1220</v>
       </c>
@@ -10289,8 +10976,11 @@
       <c r="H221">
         <v>1</v>
       </c>
-    </row>
-    <row r="222" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I221" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>1225</v>
       </c>
@@ -10315,8 +11005,11 @@
       <c r="H222">
         <v>1</v>
       </c>
-    </row>
-    <row r="223" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I222" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>1230</v>
       </c>
@@ -10341,8 +11034,11 @@
       <c r="H223">
         <v>1</v>
       </c>
-    </row>
-    <row r="224" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I223" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>1235</v>
       </c>
@@ -10367,8 +11063,11 @@
       <c r="H224">
         <v>0</v>
       </c>
-    </row>
-    <row r="225" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I224" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>1241</v>
       </c>
@@ -10393,8 +11092,11 @@
       <c r="H225">
         <v>1</v>
       </c>
-    </row>
-    <row r="226" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I225" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>1246</v>
       </c>
@@ -10419,8 +11121,11 @@
       <c r="H226">
         <v>0</v>
       </c>
-    </row>
-    <row r="227" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I226" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>1252</v>
       </c>
@@ -10445,8 +11150,11 @@
       <c r="H227">
         <v>0</v>
       </c>
-    </row>
-    <row r="228" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I227" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>1258</v>
       </c>
@@ -10471,8 +11179,11 @@
       <c r="H228">
         <v>1</v>
       </c>
-    </row>
-    <row r="229" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I228" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>1263</v>
       </c>
@@ -10497,8 +11208,11 @@
       <c r="H229">
         <v>1</v>
       </c>
-    </row>
-    <row r="230" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I229" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>1267</v>
       </c>
@@ -10523,8 +11237,11 @@
       <c r="H230">
         <v>0</v>
       </c>
-    </row>
-    <row r="231" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+      <c r="I230" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>1273</v>
       </c>
@@ -10549,8 +11266,11 @@
       <c r="H231">
         <v>1</v>
       </c>
-    </row>
-    <row r="232" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I231" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>1278</v>
       </c>
@@ -10575,8 +11295,11 @@
       <c r="H232">
         <v>0</v>
       </c>
-    </row>
-    <row r="233" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I232" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>1284</v>
       </c>
@@ -10601,8 +11324,11 @@
       <c r="H233">
         <v>1</v>
       </c>
-    </row>
-    <row r="234" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I233" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>1290</v>
       </c>
@@ -10627,8 +11353,11 @@
       <c r="H234">
         <v>1</v>
       </c>
-    </row>
-    <row r="235" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I234" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>1294</v>
       </c>
@@ -10653,34 +11382,40 @@
       <c r="H235">
         <v>1</v>
       </c>
-    </row>
-    <row r="236" spans="1:8" ht="16" x14ac:dyDescent="0.2">
-      <c r="A236" t="s">
+      <c r="I235" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A236" s="5" t="s">
         <v>1300</v>
       </c>
-      <c r="B236" s="1" t="s">
+      <c r="B236" s="6" t="s">
         <v>1301</v>
       </c>
-      <c r="C236" t="s">
+      <c r="C236" s="5" t="s">
         <v>675</v>
       </c>
-      <c r="D236" t="s">
+      <c r="D236" s="5" t="s">
         <v>1302</v>
       </c>
-      <c r="E236" s="1" t="s">
+      <c r="E236" s="6" t="s">
         <v>1303</v>
       </c>
-      <c r="F236" s="1" t="s">
+      <c r="F236" s="6" t="s">
         <v>1304</v>
       </c>
-      <c r="G236" t="s">
+      <c r="G236" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H236">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="237" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="H236" s="5" t="s">
+        <v>1390</v>
+      </c>
+      <c r="I236" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>1305</v>
       </c>
@@ -10705,8 +11440,11 @@
       <c r="H237">
         <v>1</v>
       </c>
-    </row>
-    <row r="238" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I237" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>1311</v>
       </c>
@@ -10731,8 +11469,11 @@
       <c r="H238">
         <v>1</v>
       </c>
-    </row>
-    <row r="239" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I238" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>1316</v>
       </c>
@@ -10757,8 +11498,11 @@
       <c r="H239">
         <v>1</v>
       </c>
-    </row>
-    <row r="240" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I239" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>1321</v>
       </c>
@@ -10783,8 +11527,11 @@
       <c r="H240">
         <v>1</v>
       </c>
-    </row>
-    <row r="241" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I240" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>1327</v>
       </c>
@@ -10809,8 +11556,11 @@
       <c r="H241">
         <v>0</v>
       </c>
-    </row>
-    <row r="242" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+      <c r="I241" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>1333</v>
       </c>
@@ -10835,8 +11585,11 @@
       <c r="H242">
         <v>0</v>
       </c>
-    </row>
-    <row r="243" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+      <c r="I242" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>1339</v>
       </c>
@@ -10861,8 +11614,11 @@
       <c r="H243">
         <v>1</v>
       </c>
-    </row>
-    <row r="244" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I243" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>1345</v>
       </c>
@@ -10887,8 +11643,11 @@
       <c r="H244">
         <v>0</v>
       </c>
-    </row>
-    <row r="245" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I244" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>1351</v>
       </c>
@@ -10913,8 +11672,11 @@
       <c r="H245">
         <v>1</v>
       </c>
-    </row>
-    <row r="246" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I245" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>1356</v>
       </c>
@@ -10939,8 +11701,11 @@
       <c r="H246">
         <v>0</v>
       </c>
-    </row>
-    <row r="247" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I246" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>1362</v>
       </c>
@@ -10965,8 +11730,11 @@
       <c r="H247">
         <v>1</v>
       </c>
-    </row>
-    <row r="248" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="I247" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>1367</v>
       </c>
@@ -10989,10 +11757,13 @@
         <v>14</v>
       </c>
       <c r="H248">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="249" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="I248" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>1373</v>
       </c>
@@ -11017,8 +11788,11 @@
       <c r="H249">
         <v>0</v>
       </c>
-    </row>
-    <row r="250" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+      <c r="I249" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>1379</v>
       </c>
@@ -11043,8 +11817,11 @@
       <c r="H250">
         <v>1</v>
       </c>
-    </row>
-    <row r="251" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="I250" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>1385</v>
       </c>
@@ -11067,6 +11844,9 @@
         <v>14</v>
       </c>
       <c r="H251">
+        <v>1</v>
+      </c>
+      <c r="I251" s="2">
         <v>1</v>
       </c>
     </row>

</xml_diff>